<commit_message>
feat: add MCA course structure and transcript format templates
</commit_message>
<xml_diff>
--- a/courses_data/mca_sem/MCA Course Structure Google Sheet.xlsx
+++ b/courses_data/mca_sem/MCA Course Structure Google Sheet.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="MCA Course Structure Google She" sheetId="1" r:id="rId1"/>
@@ -101,13 +101,13 @@
     <t>Discrete Mathematics</t>
   </si>
   <si>
-    <t>1MCASEC(A)</t>
+    <t>1MCASEC(C)</t>
   </si>
   <si>
     <t>Internet of Things</t>
   </si>
   <si>
-    <t>1MCASEC(C)</t>
+    <t>1MCASEC(D)</t>
   </si>
   <si>
     <t>E-Commerce</t>

</xml_diff>